<commit_message>
Final pass applied: batch 9, and health is vida everywhere
Batch 9 reviewed: the 20 keys the parser had skipped, Marine and Alien
capitalized throughout, renacer, garra, Burla, and the voice lines aligned.
Per Bleu, health is 'vida', never 'salud': the 21 lines that said salud are
swept. Glossary and style guide carry both rules. out/esES.txt: 3,854 keys,
none missing, 94% differ from English (the rest are names).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/batch9/batch9-review.xlsx
+++ b/work/batch9/batch9-review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maost\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\[01] Martin\[07] Claude Code\NS2-Spanish-Translation\work\batch9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{17787EF1-AFB7-4C84-8486-543917666811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9676D5DA-B4A0-41A2-BF65-F5955715323E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9ED70484-7489-41F5-9EA9-1A578823D461}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{9ED70484-7489-41F5-9EA9-1A578823D461}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="341">
   <si>
     <t>Section</t>
   </si>
@@ -1060,6 +1060,12 @@
   </si>
   <si>
     <t>Flagged left</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Keep current</t>
   </si>
 </sst>
 </file>
@@ -1620,7 +1626,7 @@
       </c>
       <c r="B10" s="14">
         <f>COUNTA(Review!J2:J81)</f>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -1629,7 +1635,7 @@
       </c>
       <c r="B11" s="14">
         <f>ROWS(Review!J2:J81)-COUNTA(Review!J2:J81)</f>
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -1638,7 +1644,7 @@
       </c>
       <c r="B12" s="14">
         <f>COUNTIFS(Review!G2:G81,"?*",Review!J2:J81,"")</f>
-        <v>61</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1665,7 +1671,7 @@
     <col min="12" max="12" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1723,7 +1729,9 @@
       <c r="G2" s="3"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="6"/>
+      <c r="J2" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
     </row>
@@ -1747,7 +1755,9 @@
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="6"/>
+      <c r="J3" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
     </row>
@@ -1771,7 +1781,9 @@
       <c r="G4" s="3"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="6"/>
+      <c r="J4" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
     </row>
@@ -1795,7 +1807,9 @@
       <c r="G5" s="3"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
-      <c r="J5" s="6"/>
+      <c r="J5" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
     </row>
@@ -1819,7 +1833,9 @@
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="6"/>
+      <c r="J6" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
     </row>
@@ -1843,7 +1859,9 @@
       <c r="G7" s="3"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
     </row>
@@ -1867,7 +1885,9 @@
       <c r="G8" s="3"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
     </row>
@@ -1891,7 +1911,9 @@
       <c r="G9" s="3"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="6"/>
+      <c r="J9" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
     </row>
@@ -1915,7 +1937,9 @@
       <c r="G10" s="3"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="6"/>
+      <c r="J10" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
     </row>
@@ -1941,7 +1965,9 @@
       <c r="I11" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="J11" s="6"/>
+      <c r="J11" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
     </row>
@@ -1967,7 +1993,9 @@
       <c r="I12" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="6"/>
+      <c r="J12" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
     </row>
@@ -1997,7 +2025,9 @@
       <c r="I13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J13" s="6"/>
+      <c r="J13" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
     </row>
@@ -2023,7 +2053,9 @@
       <c r="I14" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J14" s="6"/>
+      <c r="J14" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
     </row>
@@ -2049,7 +2081,9 @@
       <c r="I15" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J15" s="6"/>
+      <c r="J15" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
     </row>
@@ -2075,7 +2109,9 @@
       <c r="I16" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J16" s="6"/>
+      <c r="J16" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
     </row>
@@ -2101,7 +2137,9 @@
       <c r="I17" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J17" s="6"/>
+      <c r="J17" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
     </row>
@@ -2127,7 +2165,9 @@
       <c r="I18" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J18" s="6"/>
+      <c r="J18" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
     </row>
@@ -2153,7 +2193,9 @@
       <c r="I19" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J19" s="6"/>
+      <c r="J19" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
     </row>
@@ -2179,7 +2221,9 @@
       <c r="I20" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J20" s="6"/>
+      <c r="J20" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
     </row>
@@ -2205,7 +2249,9 @@
       <c r="I21" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J21" s="6"/>
+      <c r="J21" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K21" s="7"/>
       <c r="L21" s="7"/>
     </row>
@@ -2235,7 +2281,9 @@
         <v>85</v>
       </c>
       <c r="I22" s="4"/>
-      <c r="J22" s="6"/>
+      <c r="J22" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K22" s="7"/>
       <c r="L22" s="7"/>
     </row>
@@ -2265,7 +2313,9 @@
         <v>85</v>
       </c>
       <c r="I23" s="4"/>
-      <c r="J23" s="6"/>
+      <c r="J23" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K23" s="7"/>
       <c r="L23" s="7"/>
     </row>
@@ -2295,7 +2345,9 @@
         <v>85</v>
       </c>
       <c r="I24" s="4"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
     </row>
@@ -2325,7 +2377,9 @@
         <v>85</v>
       </c>
       <c r="I25" s="4"/>
-      <c r="J25" s="6"/>
+      <c r="J25" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
     </row>
@@ -2355,7 +2409,9 @@
         <v>85</v>
       </c>
       <c r="I26" s="4"/>
-      <c r="J26" s="6"/>
+      <c r="J26" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K26" s="7"/>
       <c r="L26" s="7"/>
     </row>
@@ -2385,7 +2441,9 @@
         <v>85</v>
       </c>
       <c r="I27" s="4"/>
-      <c r="J27" s="6"/>
+      <c r="J27" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K27" s="7"/>
       <c r="L27" s="7"/>
     </row>
@@ -2415,7 +2473,9 @@
         <v>85</v>
       </c>
       <c r="I28" s="4"/>
-      <c r="J28" s="6"/>
+      <c r="J28" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K28" s="7"/>
       <c r="L28" s="7"/>
     </row>
@@ -2445,7 +2505,9 @@
         <v>85</v>
       </c>
       <c r="I29" s="4"/>
-      <c r="J29" s="6"/>
+      <c r="J29" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K29" s="7"/>
       <c r="L29" s="7"/>
     </row>
@@ -2475,7 +2537,9 @@
         <v>85</v>
       </c>
       <c r="I30" s="4"/>
-      <c r="J30" s="6"/>
+      <c r="J30" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
     </row>
@@ -2505,7 +2569,9 @@
         <v>85</v>
       </c>
       <c r="I31" s="4"/>
-      <c r="J31" s="6"/>
+      <c r="J31" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
     </row>
@@ -2535,7 +2601,9 @@
         <v>85</v>
       </c>
       <c r="I32" s="4"/>
-      <c r="J32" s="6"/>
+      <c r="J32" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
     </row>
@@ -2565,7 +2633,9 @@
         <v>85</v>
       </c>
       <c r="I33" s="4"/>
-      <c r="J33" s="6"/>
+      <c r="J33" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
     </row>
@@ -2595,7 +2665,9 @@
         <v>85</v>
       </c>
       <c r="I34" s="4"/>
-      <c r="J34" s="6"/>
+      <c r="J34" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
     </row>
@@ -2625,7 +2697,9 @@
         <v>85</v>
       </c>
       <c r="I35" s="4"/>
-      <c r="J35" s="6"/>
+      <c r="J35" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
     </row>
@@ -2655,7 +2729,9 @@
         <v>85</v>
       </c>
       <c r="I36" s="4"/>
-      <c r="J36" s="6"/>
+      <c r="J36" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K36" s="7"/>
       <c r="L36" s="7"/>
     </row>
@@ -2685,7 +2761,9 @@
         <v>85</v>
       </c>
       <c r="I37" s="4"/>
-      <c r="J37" s="6"/>
+      <c r="J37" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
     </row>
@@ -2715,7 +2793,9 @@
         <v>85</v>
       </c>
       <c r="I38" s="4"/>
-      <c r="J38" s="6"/>
+      <c r="J38" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
     </row>
@@ -2745,7 +2825,9 @@
         <v>85</v>
       </c>
       <c r="I39" s="4"/>
-      <c r="J39" s="6"/>
+      <c r="J39" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
     </row>
@@ -2775,7 +2857,9 @@
         <v>85</v>
       </c>
       <c r="I40" s="4"/>
-      <c r="J40" s="6"/>
+      <c r="J40" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K40" s="7"/>
       <c r="L40" s="7"/>
     </row>
@@ -2805,7 +2889,9 @@
         <v>85</v>
       </c>
       <c r="I41" s="4"/>
-      <c r="J41" s="6"/>
+      <c r="J41" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
     </row>
@@ -2835,7 +2921,9 @@
         <v>85</v>
       </c>
       <c r="I42" s="4"/>
-      <c r="J42" s="6"/>
+      <c r="J42" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K42" s="7"/>
       <c r="L42" s="7"/>
     </row>
@@ -2865,7 +2953,9 @@
         <v>85</v>
       </c>
       <c r="I43" s="4"/>
-      <c r="J43" s="6"/>
+      <c r="J43" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K43" s="7"/>
       <c r="L43" s="7"/>
     </row>
@@ -2895,7 +2985,9 @@
         <v>85</v>
       </c>
       <c r="I44" s="4"/>
-      <c r="J44" s="6"/>
+      <c r="J44" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K44" s="7"/>
       <c r="L44" s="7"/>
     </row>
@@ -2925,7 +3017,9 @@
         <v>85</v>
       </c>
       <c r="I45" s="4"/>
-      <c r="J45" s="6"/>
+      <c r="J45" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K45" s="7"/>
       <c r="L45" s="7"/>
     </row>
@@ -2955,7 +3049,9 @@
         <v>85</v>
       </c>
       <c r="I46" s="4"/>
-      <c r="J46" s="6"/>
+      <c r="J46" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
     </row>
@@ -2985,7 +3081,9 @@
         <v>85</v>
       </c>
       <c r="I47" s="4"/>
-      <c r="J47" s="6"/>
+      <c r="J47" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
     </row>
@@ -3015,7 +3113,9 @@
         <v>85</v>
       </c>
       <c r="I48" s="4"/>
-      <c r="J48" s="6"/>
+      <c r="J48" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
     </row>
@@ -3045,7 +3145,9 @@
         <v>85</v>
       </c>
       <c r="I49" s="4"/>
-      <c r="J49" s="6"/>
+      <c r="J49" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K49" s="7"/>
       <c r="L49" s="7"/>
     </row>
@@ -3075,7 +3177,9 @@
         <v>85</v>
       </c>
       <c r="I50" s="4"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
     </row>
@@ -3105,7 +3209,9 @@
         <v>85</v>
       </c>
       <c r="I51" s="4"/>
-      <c r="J51" s="6"/>
+      <c r="J51" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
     </row>
@@ -3135,7 +3241,9 @@
         <v>85</v>
       </c>
       <c r="I52" s="4"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K52" s="7"/>
       <c r="L52" s="7"/>
     </row>
@@ -3165,7 +3273,9 @@
         <v>85</v>
       </c>
       <c r="I53" s="4"/>
-      <c r="J53" s="6"/>
+      <c r="J53" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K53" s="7"/>
       <c r="L53" s="7"/>
     </row>
@@ -3195,7 +3305,9 @@
         <v>85</v>
       </c>
       <c r="I54" s="4"/>
-      <c r="J54" s="6"/>
+      <c r="J54" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
     </row>
@@ -3225,7 +3337,9 @@
         <v>85</v>
       </c>
       <c r="I55" s="4"/>
-      <c r="J55" s="6"/>
+      <c r="J55" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
     </row>
@@ -3255,7 +3369,9 @@
         <v>85</v>
       </c>
       <c r="I56" s="4"/>
-      <c r="J56" s="6"/>
+      <c r="J56" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K56" s="7"/>
       <c r="L56" s="7"/>
     </row>
@@ -3285,7 +3401,9 @@
         <v>85</v>
       </c>
       <c r="I57" s="4"/>
-      <c r="J57" s="6"/>
+      <c r="J57" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K57" s="7"/>
       <c r="L57" s="7"/>
     </row>
@@ -3315,7 +3433,9 @@
         <v>85</v>
       </c>
       <c r="I58" s="4"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
     </row>
@@ -3345,7 +3465,9 @@
         <v>85</v>
       </c>
       <c r="I59" s="4"/>
-      <c r="J59" s="6"/>
+      <c r="J59" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
     </row>
@@ -3375,7 +3497,9 @@
         <v>85</v>
       </c>
       <c r="I60" s="4"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K60" s="7"/>
       <c r="L60" s="7"/>
     </row>
@@ -3405,7 +3529,9 @@
         <v>85</v>
       </c>
       <c r="I61" s="4"/>
-      <c r="J61" s="6"/>
+      <c r="J61" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K61" s="7"/>
       <c r="L61" s="7"/>
     </row>
@@ -3435,7 +3561,9 @@
         <v>85</v>
       </c>
       <c r="I62" s="4"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K62" s="7"/>
       <c r="L62" s="7"/>
     </row>
@@ -3465,7 +3593,9 @@
         <v>85</v>
       </c>
       <c r="I63" s="4"/>
-      <c r="J63" s="6"/>
+      <c r="J63" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K63" s="7"/>
       <c r="L63" s="7"/>
     </row>
@@ -3495,7 +3625,9 @@
         <v>85</v>
       </c>
       <c r="I64" s="4"/>
-      <c r="J64" s="6"/>
+      <c r="J64" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
     </row>
@@ -3525,7 +3657,9 @@
         <v>85</v>
       </c>
       <c r="I65" s="4"/>
-      <c r="J65" s="6"/>
+      <c r="J65" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
     </row>
@@ -3555,7 +3689,9 @@
         <v>85</v>
       </c>
       <c r="I66" s="4"/>
-      <c r="J66" s="6"/>
+      <c r="J66" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
     </row>
@@ -3585,7 +3721,9 @@
         <v>85</v>
       </c>
       <c r="I67" s="4"/>
-      <c r="J67" s="6"/>
+      <c r="J67" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
     </row>
@@ -3615,7 +3753,9 @@
         <v>265</v>
       </c>
       <c r="I68" s="4"/>
-      <c r="J68" s="6"/>
+      <c r="J68" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
     </row>
@@ -3645,7 +3785,9 @@
         <v>270</v>
       </c>
       <c r="I69" s="4"/>
-      <c r="J69" s="6"/>
+      <c r="J69" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
     </row>
@@ -3675,7 +3817,9 @@
         <v>274</v>
       </c>
       <c r="I70" s="4"/>
-      <c r="J70" s="6"/>
+      <c r="J70" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
     </row>
@@ -3705,7 +3849,9 @@
         <v>279</v>
       </c>
       <c r="I71" s="4"/>
-      <c r="J71" s="6"/>
+      <c r="J71" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
     </row>
@@ -3735,7 +3881,9 @@
         <v>284</v>
       </c>
       <c r="I72" s="4"/>
-      <c r="J72" s="6"/>
+      <c r="J72" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K72" s="7"/>
       <c r="L72" s="7"/>
     </row>
@@ -3765,7 +3913,9 @@
         <v>289</v>
       </c>
       <c r="I73" s="4"/>
-      <c r="J73" s="6"/>
+      <c r="J73" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K73" s="7"/>
       <c r="L73" s="7"/>
     </row>
@@ -3795,7 +3945,9 @@
         <v>294</v>
       </c>
       <c r="I74" s="4"/>
-      <c r="J74" s="6"/>
+      <c r="J74" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="K74" s="7"/>
       <c r="L74" s="7"/>
     </row>
@@ -3825,7 +3977,9 @@
         <v>299</v>
       </c>
       <c r="I75" s="4"/>
-      <c r="J75" s="6"/>
+      <c r="J75" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="K75" s="7"/>
       <c r="L75" s="7"/>
     </row>
@@ -3855,7 +4009,9 @@
         <v>304</v>
       </c>
       <c r="I76" s="4"/>
-      <c r="J76" s="6"/>
+      <c r="J76" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K76" s="7"/>
       <c r="L76" s="7"/>
     </row>
@@ -3887,7 +4043,9 @@
       <c r="I77" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="J77" s="6"/>
+      <c r="J77" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="K77" s="7"/>
       <c r="L77" s="7"/>
     </row>
@@ -3917,7 +4075,9 @@
         <v>294</v>
       </c>
       <c r="I78" s="4"/>
-      <c r="J78" s="6"/>
+      <c r="J78" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
     </row>
@@ -3947,7 +4107,9 @@
         <v>304</v>
       </c>
       <c r="I79" s="4"/>
-      <c r="J79" s="6"/>
+      <c r="J79" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
     </row>
@@ -3977,7 +4139,9 @@
         <v>294</v>
       </c>
       <c r="I80" s="4"/>
-      <c r="J80" s="6"/>
+      <c r="J80" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="K80" s="7"/>
       <c r="L80" s="7"/>
     </row>
@@ -4007,7 +4171,9 @@
         <v>294</v>
       </c>
       <c r="I81" s="4"/>
-      <c r="J81" s="6"/>
+      <c r="J81" s="6" t="s">
+        <v>340</v>
+      </c>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
     </row>

</xml_diff>